<commit_message>
Hall mark reached in analysis
</commit_message>
<xml_diff>
--- a/backend/BHT+4+SEASONS+JULY+2026.xlsx
+++ b/backend/BHT+4+SEASONS+JULY+2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Taofeek Olatunji\Documents\QC-HUB\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EFC0333-9EAE-415F-BE41-3FEF83D08717}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4F47543-CDBD-4E7F-983B-90178C8A2E56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="759" xr2:uid="{0F83F228-6889-41C6-8005-88AB2A45982A}"/>
   </bookViews>
@@ -13886,8 +13886,82 @@
     </dxf>
     <dxf>
       <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF9E004F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
         <patternFill>
           <bgColor rgb="FFE1AAA9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF6D9E"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFDCC97A"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFE4E300"/>
         </patternFill>
       </fill>
     </dxf>
@@ -13895,6 +13969,20 @@
       <fill>
         <patternFill>
           <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE1AAA9"/>
         </patternFill>
       </fill>
     </dxf>
@@ -13931,6 +14019,21 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
           <bgColor rgb="FFE4E300"/>
         </patternFill>
       </fill>
@@ -13940,6 +14043,646 @@
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
           <bgColor rgb="FFDCC97A"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="6" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF4685D2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFDCC97A"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFE4E300"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE1AAA9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF9E004F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF6D9E"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF4685D2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="6" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFBB57"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFBFB00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF852B7F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF6F626"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFE4E300"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE1AAA9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFDCC97A"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="6" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF4685D2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF6D9E"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF9E004F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFBB57"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF99BCE7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF6F626"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF852B7F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF2DBDA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF6969"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFBB57"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE1AAA9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF9E004F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF6D9E"/>
         </patternFill>
       </fill>
     </dxf>
@@ -13990,8 +14733,16 @@
     </dxf>
     <dxf>
       <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="6" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
         <patternFill>
-          <bgColor theme="7" tint="0.39994506668294322"/>
+          <bgColor rgb="FF4685D2"/>
         </patternFill>
       </fill>
     </dxf>
@@ -13999,28 +14750,14 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
-          <bgColor rgb="FF9E004F"/>
+          <bgColor theme="4" tint="0.59999389629810485"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFF6D9E"/>
+          <bgColor theme="9" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
     </dxf>
@@ -14055,7 +14792,21 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFE1AAA9"/>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9900"/>
         </patternFill>
       </fill>
     </dxf>
@@ -14127,47 +14878,10 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
       <fill>
-        <patternFill>
-          <bgColor rgb="FFFF6D9E"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE1AAA9"/>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFE4E300"/>
         </patternFill>
       </fill>
     </dxf>
@@ -14180,79 +14894,8 @@
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFE4E300"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
         <patternFill>
-          <bgColor theme="6" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="6" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF4685D2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="4" tint="0.59999389629810485"/>
+          <bgColor rgb="FFE1AAA9"/>
         </patternFill>
       </fill>
     </dxf>
@@ -14267,7 +14910,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFBB57"/>
+          <bgColor rgb="FFDDE8C6"/>
         </patternFill>
       </fill>
     </dxf>
@@ -14275,171 +14918,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
-          <bgColor rgb="FFFBFB00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF852B7F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF6F626"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFEEB400"/>
+          <bgColor rgb="FFE7D480"/>
         </patternFill>
       </fill>
     </dxf>
@@ -14454,303 +14933,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
-          <bgColor rgb="FF9E004F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE1AAA9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFE4E300"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="6" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF4685D2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="4" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFDCC97A"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF6D9E"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFBB57"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="4" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF99BCE7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF6F626"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF852B7F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF2DBDA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF6969"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFBB57"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF9E004F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF6D9E"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFE4E300"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE1AAA9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFDCC97A"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="6" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF4685D2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="4" tint="0.59999389629810485"/>
+          <bgColor rgb="FFBA005D"/>
         </patternFill>
       </fill>
     </dxf>
@@ -14758,145 +14941,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF9E004F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE1AAA9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFE4E300"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFDCC97A"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="6" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF4685D2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="4" tint="0.59999389629810485"/>
         </patternFill>
       </fill>
     </dxf>
@@ -14925,7 +14969,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
+          <bgColor theme="9" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
@@ -14933,138 +14977,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFE3E0CF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDDE8C6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFE7D480"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFBA005D"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF4685D2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="6" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFE4E300"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFDCC97A"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE1AAA9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFEEB400"/>
         </patternFill>
       </fill>
     </dxf>
@@ -15099,43 +15011,9 @@
     </dxf>
     <dxf>
       <fill>
-        <patternFill>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
-          <bgColor theme="0" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF6D9E"/>
+          <bgColor theme="6" tint="0.59999389629810485"/>
         </patternFill>
       </fill>
     </dxf>
@@ -15143,7 +15021,58 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
-          <bgColor rgb="FF9E004F"/>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFDCC97A"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFE4E300"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF4685D2"/>
         </patternFill>
       </fill>
     </dxf>
@@ -15157,7 +15086,14 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="7" tint="0.39994506668294322"/>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFEEB400"/>
         </patternFill>
       </fill>
     </dxf>
@@ -15252,6 +15188,70 @@
     </dxf>
     <dxf>
       <fill>
+        <patternFill>
+          <bgColor theme="8"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF6D9E"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF9E004F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE1AAA9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
           <bgColor theme="6" tint="0.79998168889431442"/>
@@ -15268,13 +15268,6 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFBB57"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor rgb="FFDDE8C6"/>
         </patternFill>
       </fill>
@@ -15284,6 +15277,13 @@
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
           <bgColor rgb="FFE7D480"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFBB57"/>
         </patternFill>
       </fill>
     </dxf>
@@ -15311,13 +15311,6 @@
     </dxf>
     <dxf>
       <fill>
-        <patternFill>
-          <bgColor rgb="FF99BCE7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
           <bgColor theme="4" tint="0.79998168889431442"/>
@@ -15326,9 +15319,8 @@
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="6" tint="0.79998168889431442"/>
+        <patternFill>
+          <bgColor rgb="FF99BCE7"/>
         </patternFill>
       </fill>
     </dxf>
@@ -15343,6 +15335,14 @@
       <fill>
         <patternFill>
           <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="6" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -15364,6 +15364,13 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFD44B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFBB57"/>
         </patternFill>
       </fill>
     </dxf>
@@ -15443,36 +15450,14 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFBB57"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFE4E300"/>
+          <bgColor theme="9" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="7" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF6969"/>
+          <bgColor rgb="FFFF9900"/>
         </patternFill>
       </fill>
     </dxf>
@@ -15488,9 +15473,23 @@
     </dxf>
     <dxf>
       <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
           <bgColor rgb="FFFBFB00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFEEB400"/>
         </patternFill>
       </fill>
     </dxf>
@@ -15508,7 +15507,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFEEB400"/>
+          <bgColor rgb="FFFF6969"/>
         </patternFill>
       </fill>
     </dxf>
@@ -15522,21 +15521,14 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFF9900"/>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
+          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -15544,7 +15536,23 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
-          <bgColor theme="4" tint="0.59999389629810485"/>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFE4E300"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="6" tint="0.59999389629810485"/>
         </patternFill>
       </fill>
     </dxf>
@@ -15559,29 +15567,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
-          <bgColor theme="6" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.24994659260841701"/>
+          <bgColor theme="4" tint="0.59999389629810485"/>
         </patternFill>
       </fill>
     </dxf>
@@ -15597,6 +15583,20 @@
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
           <bgColor rgb="FFDCC97A"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8"/>
         </patternFill>
       </fill>
     </dxf>
@@ -15626,6 +15626,20 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -15674,13 +15688,6 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor theme="0" tint="-0.14996795556505021"/>
         </patternFill>
       </fill>
@@ -15688,210 +15695,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
@@ -15947,7 +15751,70 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -15968,7 +15835,28 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
@@ -15983,20 +15871,6 @@
       <fill>
         <patternFill>
           <bgColor theme="6" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
@@ -16031,7 +15905,14 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="6" tint="0.39994506668294322"/>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
@@ -16045,7 +15926,126 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
         </patternFill>
       </fill>
     </dxf>
@@ -16080,6 +16080,20 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor theme="3" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor theme="6" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
@@ -16087,7 +16101,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
+          <bgColor theme="5" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
@@ -16108,27 +16122,6 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor theme="3" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
@@ -16136,7 +16129,42 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="6" tint="0.39994506668294322"/>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -16147,6 +16175,28 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFF6D9E"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF9E004F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
         </patternFill>
       </fill>
     </dxf>
@@ -16185,15 +16235,16 @@
     </dxf>
     <dxf>
       <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.24994659260841701"/>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFDCC97A"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFF0000"/>
+          <bgColor theme="6" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
     </dxf>
@@ -16230,41 +16281,6 @@
     </dxf>
     <dxf>
       <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
           <bgColor rgb="FF9E004F"/>
@@ -16273,9 +16289,8 @@
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFDCC97A"/>
+        <patternFill>
+          <bgColor rgb="FFE1AAA9"/>
         </patternFill>
       </fill>
     </dxf>
@@ -16303,22 +16318,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFE1AAA9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF9E004F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.59996337778862885"/>
+          <bgColor theme="3" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -16326,6 +16326,27 @@
       <fill>
         <patternFill>
           <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -16346,14 +16367,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
+          <bgColor theme="3" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
@@ -16367,36 +16381,14 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="3" tint="0.79998168889431442"/>
+          <bgColor theme="6" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFDCC97A"/>
+          <bgColor theme="7" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
     </dxf>
@@ -16410,15 +16402,9 @@
     </dxf>
     <dxf>
       <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF9900"/>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="6" tint="0.59999389629810485"/>
         </patternFill>
       </fill>
     </dxf>
@@ -16426,34 +16412,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FF4685D2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFEEB400"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
     </dxf>
@@ -16469,7 +16427,49 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
-          <bgColor theme="6" tint="0.59999389629810485"/>
+          <bgColor rgb="FFDCC97A"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFEEB400"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFEEB400"/>
         </patternFill>
       </fill>
     </dxf>
@@ -48708,7 +48708,7 @@
       </c>
       <c r="O1599" s="2" t="str">
         <f ca="1">TEXT(YEAR(NOW())-2000, "00") &amp; TEXT(MONTH(NOW()), "00") &amp; TEXT(DAY(NOW()), "00") &amp; TEXT(HOUR(NOW()), "00") &amp; TEXT(MINUTE(NOW()), "00")</f>
-        <v>2608021940</v>
+        <v>2608040700</v>
       </c>
     </row>
   </sheetData>
@@ -48721,172 +48721,172 @@
     <cfRule type="expression" dxfId="349" priority="141" stopIfTrue="1">
       <formula>OR($A1598="username", $A1598="phonenumber", $A1598="start", $A1598="end", $A1598="deviceid", $A1598="subscriberid", $A1598="simserial", $A1598="caseid")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="348" priority="142" stopIfTrue="1">
-      <formula>OR(AND(LEFT($A1598, 16)="select_multiple ", LEN($A1598)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A1598, 17)))), AND(LEFT($A1598, 11)="select_one ", LEN($A1598)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A1598, 12)))))</formula>
+    <cfRule type="expression" dxfId="348" priority="149" stopIfTrue="1">
+      <formula>$A1598="begin group"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="347" priority="144" stopIfTrue="1">
-      <formula>$A1598="integer"</formula>
+    <cfRule type="expression" dxfId="347" priority="148" stopIfTrue="1">
+      <formula>$A1598="end group"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="346" priority="145" stopIfTrue="1">
-      <formula>$A1598="text"</formula>
+    <cfRule type="expression" dxfId="346" priority="139" stopIfTrue="1">
+      <formula>OR($A1598="geopoint", $A1598="geoshape", $A1598="geotrace")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="345" priority="147" stopIfTrue="1">
       <formula>$A1598="begin repeat"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="344" priority="148" stopIfTrue="1">
-      <formula>$A1598="end group"</formula>
+    <cfRule type="expression" dxfId="344" priority="146" stopIfTrue="1">
+      <formula>$A1598="end repeat"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="343" priority="149" stopIfTrue="1">
-      <formula>$A1598="begin group"</formula>
+    <cfRule type="expression" dxfId="343" priority="145" stopIfTrue="1">
+      <formula>$A1598="text"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="342" priority="143" stopIfTrue="1">
+    <cfRule type="expression" dxfId="342" priority="137" stopIfTrue="1">
+      <formula>$A1598="note"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="341" priority="144" stopIfTrue="1">
+      <formula>$A1598="integer"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="340" priority="143" stopIfTrue="1">
       <formula>$A1598="decimal"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="341" priority="146" stopIfTrue="1">
-      <formula>$A1598="end repeat"</formula>
+    <cfRule type="expression" dxfId="339" priority="142" stopIfTrue="1">
+      <formula>OR(AND(LEFT($A1598, 16)="select_multiple ", LEN($A1598)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A1598, 17)))), AND(LEFT($A1598, 11)="select_one ", LEN($A1598)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A1598, 12)))))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="340" priority="135" stopIfTrue="1">
+    <cfRule type="expression" dxfId="338" priority="136" stopIfTrue="1">
+      <formula>OR($A1598="calculate", $A1598="calculate_here")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="337" priority="135" stopIfTrue="1">
       <formula>OR($A1598="date", $A1598="datetime")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="339" priority="136" stopIfTrue="1">
-      <formula>OR($A1598="calculate", $A1598="calculate_here")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="338" priority="137" stopIfTrue="1">
-      <formula>$A1598="note"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="337" priority="138" stopIfTrue="1">
+    <cfRule type="expression" dxfId="336" priority="138" stopIfTrue="1">
       <formula>$A1598="barcode"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="336" priority="139" stopIfTrue="1">
-      <formula>OR($A1598="geopoint", $A1598="geoshape", $A1598="geotrace")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A840:B842 D840:X842 A1566:X1596">
-    <cfRule type="expression" dxfId="335" priority="569">
+    <cfRule type="expression" dxfId="335" priority="568">
+      <formula>$A840="begin group"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="334" priority="570">
+      <formula>AND(LEFT($A840,15)="select_multiple",LEN($A840)&gt;14)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="333" priority="564">
+      <formula>$A840="text"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="332" priority="563">
+      <formula>$A840="type"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="331" priority="569">
       <formula>$A840="note"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="334" priority="571">
-      <formula>AND(LEFT($A840, 10)="select_one", LEN($A840)&gt;9)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="333" priority="568">
-      <formula>$A840="begin group"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="332" priority="566">
-      <formula>$A840="integer"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="331" priority="565">
+    <cfRule type="expression" dxfId="330" priority="565">
       <formula>$A840="calculate"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="330" priority="564">
-      <formula>$A840="text"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="329" priority="563">
-      <formula>$A840="type"</formula>
+    <cfRule type="expression" dxfId="329" priority="566">
+      <formula>$A840="integer"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="328" priority="567">
       <formula>$A840="end group"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="327" priority="570">
-      <formula>AND(LEFT($A840,15)="select_multiple",LEN($A840)&gt;14)</formula>
+    <cfRule type="expression" dxfId="327" priority="571">
+      <formula>AND(LEFT($A840, 10)="select_one", LEN($A840)&gt;9)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1598:B1598">
-    <cfRule type="expression" dxfId="326" priority="101" stopIfTrue="1">
-      <formula>OR($A1598="audio", $A1598="video")</formula>
+    <cfRule type="expression" dxfId="326" priority="99" stopIfTrue="1">
+      <formula>$A1598="comments"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="325" priority="102" stopIfTrue="1">
+    <cfRule type="expression" dxfId="325" priority="98" stopIfTrue="1">
+      <formula>OR(AND(LEFT($A1598, 14)="sensor_stream ", LEN($A1598)&gt;14, NOT(ISNUMBER(SEARCH(" ", $A1598, 15)))), AND(LEFT($A1598, 17)="sensor_statistic ", LEN($A1598)&gt;17, NOT(ISNUMBER(SEARCH(" ", $A1598, 18)))))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="324" priority="102" stopIfTrue="1">
       <formula>$A1598="image"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="324" priority="99" stopIfTrue="1">
-      <formula>$A1598="comments"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="323" priority="98" stopIfTrue="1">
-      <formula>OR(AND(LEFT($A1598, 14)="sensor_stream ", LEN($A1598)&gt;14, NOT(ISNUMBER(SEARCH(" ", $A1598, 15)))), AND(LEFT($A1598, 17)="sensor_statistic ", LEN($A1598)&gt;17, NOT(ISNUMBER(SEARCH(" ", $A1598, 18)))))</formula>
+    <cfRule type="expression" dxfId="323" priority="101" stopIfTrue="1">
+      <formula>OR($A1598="audio", $A1598="video")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1565:D1565 F1565:J1565 L1565:P1565 R1565:W1565">
-    <cfRule type="expression" dxfId="322" priority="324" stopIfTrue="1">
+    <cfRule type="expression" dxfId="322" priority="331" stopIfTrue="1">
+      <formula>$A1565="integer"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="321" priority="330" stopIfTrue="1">
+      <formula>$A1565="decimal"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="320" priority="329" stopIfTrue="1">
+      <formula>OR(AND(LEFT($A1565, 16)="select_multiple ", LEN($A1565)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A1565, 17)))), AND(LEFT($A1565, 11)="select_one ", LEN($A1565)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A1565, 12)))))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="319" priority="328" stopIfTrue="1">
+      <formula>OR($A1565="username", $A1565="phonenumber", $A1565="start", $A1565="end", $A1565="deviceid", $A1565="subscriberid", $A1565="simserial", $A1565="caseid")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="318" priority="325" stopIfTrue="1">
+      <formula>$A1565="barcode"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="317" priority="324" stopIfTrue="1">
       <formula>$A1565="note"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="321" priority="337" stopIfTrue="1">
+    <cfRule type="expression" dxfId="316" priority="323" stopIfTrue="1">
+      <formula>OR($A1565="calculate", $A1565="calculate_here")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="315" priority="322" stopIfTrue="1">
+      <formula>OR($A1565="date", $A1565="datetime")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="314" priority="321" stopIfTrue="1">
+      <formula>$A1565="image"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="313" priority="320" stopIfTrue="1">
+      <formula>$A1565="comments"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="312" priority="326" stopIfTrue="1">
+      <formula>OR($A1565="geopoint", $A1565="geoshape", $A1565="geotrace")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="311" priority="337" stopIfTrue="1">
       <formula>OR($A1565="audio", $A1565="video")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="320" priority="336" stopIfTrue="1">
+    <cfRule type="expression" dxfId="310" priority="336" stopIfTrue="1">
       <formula>$A1565="begin group"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="319" priority="335" stopIfTrue="1">
+    <cfRule type="expression" dxfId="309" priority="319" stopIfTrue="1">
+      <formula>OR(AND(LEFT($A1565, 14)="sensor_stream ", LEN($A1565)&gt;14, NOT(ISNUMBER(SEARCH(" ", $A1565, 15)))), AND(LEFT($A1565, 17)="sensor_statistic ", LEN($A1565)&gt;17, NOT(ISNUMBER(SEARCH(" ", $A1565, 18)))))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="308" priority="327" stopIfTrue="1">
+      <formula>OR($A1565="audio audit", $A1565="text audit", $A1565="speed violations count", $A1565="speed violations list", $A1565="speed violations audit")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="307" priority="335" stopIfTrue="1">
       <formula>$A1565="end group"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="318" priority="334" stopIfTrue="1">
+    <cfRule type="expression" dxfId="306" priority="334" stopIfTrue="1">
       <formula>$A1565="begin repeat"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="317" priority="333" stopIfTrue="1">
+    <cfRule type="expression" dxfId="305" priority="333" stopIfTrue="1">
       <formula>$A1565="end repeat"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="316" priority="332" stopIfTrue="1">
+    <cfRule type="expression" dxfId="304" priority="332" stopIfTrue="1">
       <formula>$A1565="text"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="315" priority="331" stopIfTrue="1">
-      <formula>$A1565="integer"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="314" priority="330" stopIfTrue="1">
-      <formula>$A1565="decimal"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="313" priority="329" stopIfTrue="1">
-      <formula>OR(AND(LEFT($A1565, 16)="select_multiple ", LEN($A1565)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A1565, 17)))), AND(LEFT($A1565, 11)="select_one ", LEN($A1565)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A1565, 12)))))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="312" priority="328" stopIfTrue="1">
-      <formula>OR($A1565="username", $A1565="phonenumber", $A1565="start", $A1565="end", $A1565="deviceid", $A1565="subscriberid", $A1565="simserial", $A1565="caseid")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="311" priority="327" stopIfTrue="1">
-      <formula>OR($A1565="audio audit", $A1565="text audit", $A1565="speed violations count", $A1565="speed violations list", $A1565="speed violations audit")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="310" priority="326" stopIfTrue="1">
-      <formula>OR($A1565="geopoint", $A1565="geoshape", $A1565="geotrace")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="309" priority="323" stopIfTrue="1">
-      <formula>OR($A1565="calculate", $A1565="calculate_here")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="308" priority="322" stopIfTrue="1">
-      <formula>OR($A1565="date", $A1565="datetime")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="307" priority="321" stopIfTrue="1">
-      <formula>$A1565="image"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="306" priority="320" stopIfTrue="1">
-      <formula>$A1565="comments"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="305" priority="319" stopIfTrue="1">
-      <formula>OR(AND(LEFT($A1565, 14)="sensor_stream ", LEN($A1565)&gt;14, NOT(ISNUMBER(SEARCH(" ", $A1565, 15)))), AND(LEFT($A1565, 17)="sensor_statistic ", LEN($A1565)&gt;17, NOT(ISNUMBER(SEARCH(" ", $A1565, 18)))))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="304" priority="325" stopIfTrue="1">
-      <formula>$A1565="barcode"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1508:H1508 K1508 A1509:K1509 A1528:K1530 A1531:H1531 K1531 A1597:K1597 A1605:X1048576">
-    <cfRule type="expression" dxfId="303" priority="638">
+    <cfRule type="expression" dxfId="303" priority="631">
+      <formula>$A1508="text"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="302" priority="638">
       <formula>AND(LEFT($A1508, 10)="select_one", LEN($A1508)&gt;9)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="302" priority="634">
+    <cfRule type="expression" dxfId="301" priority="633">
+      <formula>$A1508="integer"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="300" priority="632">
+      <formula>$A1508="calculate"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="299" priority="634">
       <formula>$A1508="end group"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="301" priority="637">
-      <formula>AND(LEFT($A1508,15)="select_multiple",LEN($A1508)&gt;14)</formula>
+    <cfRule type="expression" dxfId="298" priority="635">
+      <formula>$A1508="begin group"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="300" priority="636">
+    <cfRule type="expression" dxfId="297" priority="636">
       <formula>$A1508="note"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="299" priority="633">
-      <formula>$A1508="integer"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="298" priority="632">
-      <formula>$A1508="calculate"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="297" priority="631">
-      <formula>$A1508="text"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="296" priority="635">
-      <formula>$A1508="begin group"</formula>
+    <cfRule type="expression" dxfId="296" priority="637">
+      <formula>AND(LEFT($A1508,15)="select_multiple",LEN($A1508)&gt;14)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1597:K1597 A1508:H1508 K1508 A1509:K1509 A1528:K1530 A1531:H1531 K1531 A1605:X1048576">
@@ -48904,11 +48904,11 @@
     <cfRule type="expression" dxfId="292" priority="205">
       <formula>$A1551="integer"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="291" priority="206">
+    <cfRule type="expression" dxfId="291" priority="211">
+      <formula>$A1551="type"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="290" priority="206">
       <formula>$A1551="end group"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="290" priority="211">
-      <formula>$A1551="type"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="289" priority="207">
       <formula>$A1551="begin group"</formula>
@@ -48916,185 +48916,185 @@
     <cfRule type="expression" dxfId="288" priority="208">
       <formula>$A1551="note"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="287" priority="210">
+    <cfRule type="expression" dxfId="287" priority="209">
+      <formula>AND(LEFT($A1551,15)="select_multiple",LEN($A1551)&gt;14)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="286" priority="210">
       <formula>AND(LEFT($A1551, 10)="select_one", LEN($A1551)&gt;9)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="286" priority="209">
-      <formula>AND(LEFT($A1551,15)="select_multiple",LEN($A1551)&gt;14)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1558:W1560">
-    <cfRule type="expression" dxfId="285" priority="190">
+    <cfRule type="expression" dxfId="285" priority="194">
+      <formula>$A1558="text"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="284" priority="190">
       <formula>$A1558="note"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="284" priority="187">
-      <formula>$A1558="integer"</formula>
+    <cfRule type="expression" dxfId="283" priority="191">
+      <formula>AND(LEFT($A1558,15)="select_multiple",LEN($A1558)&gt;14)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="283" priority="186">
+    <cfRule type="expression" dxfId="282" priority="192">
+      <formula>AND(LEFT($A1558, 10)="select_one", LEN($A1558)&gt;9)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="281" priority="193">
+      <formula>$A1558="type"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="280" priority="188">
+      <formula>$A1558="end group"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="279" priority="189">
+      <formula>$A1558="begin group"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="278" priority="186">
       <formula>$A1558="calculate"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="282" priority="189">
-      <formula>$A1558="begin group"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="281" priority="188">
-      <formula>$A1558="end group"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="280" priority="193">
-      <formula>$A1558="type"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="279" priority="192">
-      <formula>AND(LEFT($A1558, 10)="select_one", LEN($A1558)&gt;9)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="278" priority="191">
-      <formula>AND(LEFT($A1558,15)="select_multiple",LEN($A1558)&gt;14)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="277" priority="194">
-      <formula>$A1558="text"</formula>
+    <cfRule type="expression" dxfId="277" priority="187">
+      <formula>$A1558="integer"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:X839 A1504:K1507 L1504:X1509 A1532:X1550 A1552:X1557 A1561:X1564">
-    <cfRule type="expression" dxfId="276" priority="547">
+    <cfRule type="expression" dxfId="276" priority="550">
+      <formula>$A1="begin group"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="275" priority="547">
       <formula>$A1="calculate"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="275" priority="546">
+    <cfRule type="expression" dxfId="274" priority="546">
       <formula>$A1="text"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="274" priority="545">
+    <cfRule type="expression" dxfId="273" priority="545">
       <formula>$A1="type"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="273" priority="553">
+    <cfRule type="expression" dxfId="272" priority="548">
+      <formula>$A1="integer"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="271" priority="549">
+      <formula>$A1="end group"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="270" priority="551">
+      <formula>$A1="note"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="269" priority="553">
       <formula>AND(LEFT($A1, 10)="select_one", LEN($A1)&gt;9)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="272" priority="552">
+    <cfRule type="expression" dxfId="268" priority="552">
       <formula>AND(LEFT($A1,15)="select_multiple",LEN($A1)&gt;14)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="271" priority="551">
-      <formula>$A1="note"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="270" priority="550">
-      <formula>$A1="begin group"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="269" priority="548">
-      <formula>$A1="integer"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="268" priority="549">
-      <formula>$A1="end group"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A843:X1503">
-    <cfRule type="expression" dxfId="267" priority="352">
+    <cfRule type="expression" dxfId="267" priority="353">
+      <formula>$A843="note"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="266" priority="352">
       <formula>$A843="begin group"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="266" priority="353">
-      <formula>$A843="note"</formula>
+    <cfRule type="expression" dxfId="265" priority="351">
+      <formula>$A843="end group"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="265" priority="354">
-      <formula>AND(LEFT($A843,15)="select_multiple",LEN($A843)&gt;14)</formula>
+    <cfRule type="expression" dxfId="264" priority="350">
+      <formula>$A843="integer"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="264" priority="347">
+    <cfRule type="expression" dxfId="263" priority="349">
+      <formula>$A843="calculate"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="262" priority="347">
       <formula>$A843="type"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="263" priority="348">
+    <cfRule type="expression" dxfId="261" priority="348">
       <formula>$A843="text"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="262" priority="355">
+    <cfRule type="expression" dxfId="260" priority="355">
       <formula>AND(LEFT($A843, 10)="select_one", LEN($A843)&gt;9)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="261" priority="349">
-      <formula>$A843="calculate"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="260" priority="350">
-      <formula>$A843="integer"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="259" priority="351">
-      <formula>$A843="end group"</formula>
+    <cfRule type="expression" dxfId="259" priority="354">
+      <formula>AND(LEFT($A843,15)="select_multiple",LEN($A843)&gt;14)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1510:X1527">
-    <cfRule type="expression" dxfId="258" priority="261">
+    <cfRule type="expression" dxfId="258" priority="260">
+      <formula>$A1510="calculate"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="257" priority="258">
+      <formula>$A1510="type"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="256" priority="261">
       <formula>$A1510="integer"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="257" priority="260">
-      <formula>$A1510="calculate"</formula>
+    <cfRule type="expression" dxfId="255" priority="262">
+      <formula>$A1510="end group"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="256" priority="259">
+    <cfRule type="expression" dxfId="254" priority="259">
       <formula>$A1510="text"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="255" priority="265">
-      <formula>AND(LEFT($A1510,15)="select_multiple",LEN($A1510)&gt;14)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="254" priority="266">
-      <formula>AND(LEFT($A1510, 10)="select_one", LEN($A1510)&gt;9)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="253" priority="262">
-      <formula>$A1510="end group"</formula>
+    <cfRule type="expression" dxfId="253" priority="263">
+      <formula>$A1510="begin group"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="252" priority="264">
       <formula>$A1510="note"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="251" priority="263">
-      <formula>$A1510="begin group"</formula>
+    <cfRule type="expression" dxfId="251" priority="265">
+      <formula>AND(LEFT($A1510,15)="select_multiple",LEN($A1510)&gt;14)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="250" priority="258">
-      <formula>$A1510="type"</formula>
+    <cfRule type="expression" dxfId="250" priority="266">
+      <formula>AND(LEFT($A1510, 10)="select_one", LEN($A1510)&gt;9)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1599:X1600">
-    <cfRule type="expression" dxfId="249" priority="648">
+    <cfRule type="expression" dxfId="249" priority="651">
+      <formula>$A1599="integer"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="248" priority="650">
+      <formula>$A1599="calculate"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="247" priority="649">
+      <formula>$A1599="text"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="246" priority="648">
       <formula>$A1599="type"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="248" priority="649">
-      <formula>$A1599="text"</formula>
+    <cfRule type="expression" dxfId="245" priority="656">
+      <formula>AND(LEFT($A1599, 10)="select_one", LEN($A1599)&gt;9)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="247" priority="650">
-      <formula>$A1599="calculate"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="246" priority="651">
-      <formula>$A1599="integer"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="245" priority="652">
-      <formula>$A1599="end group"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="244" priority="653">
-      <formula>$A1599="begin group"</formula>
+    <cfRule type="expression" dxfId="244" priority="655">
+      <formula>AND(LEFT($A1599,15)="select_multiple",LEN($A1599)&gt;14)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="243" priority="654">
       <formula>$A1599="note"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="242" priority="655">
-      <formula>AND(LEFT($A1599,15)="select_multiple",LEN($A1599)&gt;14)</formula>
+    <cfRule type="expression" dxfId="242" priority="653">
+      <formula>$A1599="begin group"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="241" priority="656">
-      <formula>AND(LEFT($A1599, 10)="select_one", LEN($A1599)&gt;9)</formula>
+    <cfRule type="expression" dxfId="241" priority="652">
+      <formula>$A1599="end group"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1602:X1603">
-    <cfRule type="expression" dxfId="240" priority="2619">
-      <formula>$A1602="type"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="239" priority="2620">
+    <cfRule type="expression" dxfId="240" priority="2620">
       <formula>$A1602="text"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="238" priority="2621">
+    <cfRule type="expression" dxfId="239" priority="2622">
+      <formula>$A1602="integer"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="238" priority="2623">
+      <formula>$A1602="end group"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="237" priority="2624">
+      <formula>$A1602="begin group"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="236" priority="2625">
+      <formula>$A1602="note"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="235" priority="2626">
+      <formula>AND(LEFT($A1602,15)="select_multiple",LEN($A1602)&gt;14)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="234" priority="2627">
+      <formula>AND(LEFT($A1602, 10)="select_one", LEN($A1602)&gt;9)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="233" priority="2621">
       <formula>$A1602="calculate"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="237" priority="2622">
-      <formula>$A1602="integer"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="236" priority="2623">
-      <formula>$A1602="end group"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="235" priority="2624">
-      <formula>$A1602="begin group"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="234" priority="2625">
-      <formula>$A1602="note"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="233" priority="2626">
-      <formula>AND(LEFT($A1602,15)="select_multiple",LEN($A1602)&gt;14)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="232" priority="2627">
-      <formula>AND(LEFT($A1602, 10)="select_one", LEN($A1602)&gt;9)</formula>
+    <cfRule type="expression" dxfId="232" priority="2619">
+      <formula>$A1602="type"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1565 F1565:G1565 E1598 G1598">
@@ -49113,100 +49113,100 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1598">
-    <cfRule type="expression" dxfId="228" priority="105" stopIfTrue="1">
+    <cfRule type="expression" dxfId="228" priority="100" stopIfTrue="1">
+      <formula>$A1598="enumerator"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="227" priority="103" stopIfTrue="1">
+      <formula>OR($A1598="date", $A1598="datetime", $A1598="time")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="226" priority="105" stopIfTrue="1">
       <formula>$A1598="note"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="227" priority="106" stopIfTrue="1">
+    <cfRule type="expression" dxfId="225" priority="106" stopIfTrue="1">
       <formula>$A1598="barcode"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="226" priority="107" stopIfTrue="1">
+    <cfRule type="expression" dxfId="224" priority="112" stopIfTrue="1">
+      <formula>$A1598="integer"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="223" priority="111" stopIfTrue="1">
+      <formula>$A1598="decimal"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="222" priority="110" stopIfTrue="1">
+      <formula>OR(AND(LEFT($A1598, 16)="select_multiple ", LEN($A1598)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A1598, 17)))), AND(LEFT($A1598, 11)="select_one ", LEN($A1598)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A1598, 12)))))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="221" priority="104" stopIfTrue="1">
+      <formula>OR($A1598="calculate", $A1598="calculate_here")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="220" priority="109" stopIfTrue="1">
+      <formula>OR($A1598="username", $A1598="phonenumber", $A1598="start", $A1598="end", $A1598="deviceid", $A1598="subscriberid", $A1598="simserial", $A1598="caseid")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="219" priority="108" stopIfTrue="1">
+      <formula>OR($A1598="audio audit", $A1598="text audit", $A1598="speed violations count", $A1598="speed violations list", $A1598="speed violations audit")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="218" priority="107" stopIfTrue="1">
       <formula>OR($A1598="geopoint", $A1598="geoshape", $A1598="geotrace")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="225" priority="108" stopIfTrue="1">
+    <cfRule type="expression" dxfId="217" priority="117" stopIfTrue="1">
+      <formula>$A1598="begin group"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="216" priority="121" stopIfTrue="1">
       <formula>OR($A1598="audio audit", $A1598="text audit", $A1598="speed violations count", $A1598="speed violations list", $A1598="speed violations audit")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="224" priority="109" stopIfTrue="1">
-      <formula>OR($A1598="username", $A1598="phonenumber", $A1598="start", $A1598="end", $A1598="deviceid", $A1598="subscriberid", $A1598="simserial", $A1598="caseid")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="223" priority="110" stopIfTrue="1">
-      <formula>OR(AND(LEFT($A1598, 16)="select_multiple ", LEN($A1598)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A1598, 17)))), AND(LEFT($A1598, 11)="select_one ", LEN($A1598)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A1598, 12)))))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="222" priority="111" stopIfTrue="1">
-      <formula>$A1598="decimal"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="221" priority="112" stopIfTrue="1">
-      <formula>$A1598="integer"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="220" priority="113" stopIfTrue="1">
-      <formula>$A1598="text"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="219" priority="114" stopIfTrue="1">
-      <formula>$A1598="end repeat"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="218" priority="115" stopIfTrue="1">
-      <formula>$A1598="begin repeat"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="217" priority="116" stopIfTrue="1">
-      <formula>$A1598="end group"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="216" priority="117" stopIfTrue="1">
-      <formula>$A1598="begin group"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="215" priority="118" stopIfTrue="1">
       <formula>$A1598="comments"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="214" priority="119" stopIfTrue="1">
+    <cfRule type="expression" dxfId="214" priority="116" stopIfTrue="1">
+      <formula>$A1598="end group"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="213" priority="119" stopIfTrue="1">
       <formula>OR($A1598="calculate", $A1598="calculate_here")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="213" priority="120" stopIfTrue="1">
+    <cfRule type="expression" dxfId="212" priority="115" stopIfTrue="1">
+      <formula>$A1598="begin repeat"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="211" priority="120" stopIfTrue="1">
       <formula>OR(AND(LEFT($A1598, 14)="sensor_stream ", LEN($A1598)&gt;14, NOT(ISNUMBER(SEARCH(" ", $A1598, 15)))), AND(LEFT($A1598, 17)="sensor_statistic ", LEN($A1598)&gt;17, NOT(ISNUMBER(SEARCH(" ", $A1598, 18)))))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="212" priority="121" stopIfTrue="1">
-      <formula>OR($A1598="audio audit", $A1598="text audit", $A1598="speed violations count", $A1598="speed violations list", $A1598="speed violations audit")</formula>
+    <cfRule type="expression" dxfId="210" priority="114" stopIfTrue="1">
+      <formula>$A1598="end repeat"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="211" priority="100" stopIfTrue="1">
-      <formula>$A1598="enumerator"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="210" priority="103" stopIfTrue="1">
-      <formula>OR($A1598="date", $A1598="datetime", $A1598="time")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="209" priority="104" stopIfTrue="1">
-      <formula>OR($A1598="calculate", $A1598="calculate_here")</formula>
+    <cfRule type="expression" dxfId="209" priority="113" stopIfTrue="1">
+      <formula>$A1598="text"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1598:C1598">
-    <cfRule type="expression" dxfId="208" priority="90" stopIfTrue="1">
-      <formula>$A1598="begin repeat"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="207" priority="80" stopIfTrue="1">
+    <cfRule type="expression" dxfId="208" priority="80" stopIfTrue="1">
       <formula>$A1598="file"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="206" priority="81" stopIfTrue="1">
+    <cfRule type="expression" dxfId="207" priority="81" stopIfTrue="1">
       <formula>OR($A1598="audio", $A1598="video")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="205" priority="82" stopIfTrue="1">
+    <cfRule type="expression" dxfId="206" priority="82" stopIfTrue="1">
       <formula>$A1598="note"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="204" priority="83" stopIfTrue="1">
+    <cfRule type="expression" dxfId="205" priority="83" stopIfTrue="1">
       <formula>$A1598="barcode"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="203" priority="84" stopIfTrue="1">
+    <cfRule type="expression" dxfId="204" priority="84" stopIfTrue="1">
       <formula>OR($A1598="geopoint", $A1598="geoshape", $A1598="geotrace")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="202" priority="85" stopIfTrue="1">
+    <cfRule type="expression" dxfId="203" priority="85" stopIfTrue="1">
       <formula>$A1598="file"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="201" priority="86" stopIfTrue="1">
+    <cfRule type="expression" dxfId="202" priority="86" stopIfTrue="1">
       <formula>$A1598="decimal"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="200" priority="87" stopIfTrue="1">
+    <cfRule type="expression" dxfId="201" priority="87" stopIfTrue="1">
       <formula>$A1598="integer"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="199" priority="88" stopIfTrue="1">
+    <cfRule type="expression" dxfId="200" priority="88" stopIfTrue="1">
       <formula>$A1598="enumerator"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="198" priority="92" stopIfTrue="1">
+    <cfRule type="expression" dxfId="199" priority="92" stopIfTrue="1">
       <formula>OR($A1598="date", $A1598="datetime", $A1598="time")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="198" priority="90" stopIfTrue="1">
+      <formula>$A1598="begin repeat"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="197" priority="94" stopIfTrue="1">
       <formula>$A1598="begin group"</formula>
@@ -49219,22 +49219,22 @@
     <cfRule type="expression" dxfId="195" priority="287" stopIfTrue="1">
       <formula>$A1565="text"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="194" priority="311" stopIfTrue="1">
+    <cfRule type="expression" dxfId="194" priority="312" stopIfTrue="1">
+      <formula>OR(AND(LEFT($A1565, 16)="select_multiple ", LEN($A1565)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A1565, 17)))), AND(LEFT($A1565, 11)="select_one ", LEN($A1565)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A1565, 12)))))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="193" priority="311" stopIfTrue="1">
       <formula>OR($A1565="date", $A1565="datetime")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="193" priority="313" stopIfTrue="1">
+    <cfRule type="expression" dxfId="192" priority="313" stopIfTrue="1">
       <formula>$A1565="image"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="192" priority="312" stopIfTrue="1">
-      <formula>OR(AND(LEFT($A1565, 16)="select_multiple ", LEN($A1565)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A1565, 17)))), AND(LEFT($A1565, 11)="select_one ", LEN($A1565)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A1565, 12)))))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1565:D1565 H1565:I1565">
-    <cfRule type="expression" dxfId="191" priority="315" stopIfTrue="1">
+    <cfRule type="expression" dxfId="191" priority="314" stopIfTrue="1">
+      <formula>$A1565="decimal"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="190" priority="315" stopIfTrue="1">
       <formula>$A1565="integer"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="190" priority="314" stopIfTrue="1">
-      <formula>$A1565="decimal"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1565:D1565 J1565 F1565:G1565 E1598 G1598">
@@ -49249,14 +49249,14 @@
     <cfRule type="expression" dxfId="187" priority="308" stopIfTrue="1">
       <formula>OR($A1565="geopoint", $A1565="geoshape", $A1565="geotrace")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="186" priority="306" stopIfTrue="1">
+    <cfRule type="expression" dxfId="186" priority="305" stopIfTrue="1">
+      <formula>$A1565="begin repeat"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="185" priority="306" stopIfTrue="1">
       <formula>$A1565="note"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="185" priority="307" stopIfTrue="1">
+    <cfRule type="expression" dxfId="184" priority="307" stopIfTrue="1">
       <formula>$A1565="barcode"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="184" priority="305" stopIfTrue="1">
-      <formula>$A1565="begin repeat"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1598:D1598">
@@ -49268,192 +49268,192 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1598">
-    <cfRule type="expression" dxfId="181" priority="77" stopIfTrue="1">
+    <cfRule type="expression" dxfId="181" priority="78" stopIfTrue="1">
+      <formula>$A1598="end group"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="180" priority="65" stopIfTrue="1">
+      <formula>OR($A1598="date", $A1598="datetime", $A1598="time")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="179" priority="64" stopIfTrue="1">
+      <formula>$A1598="image"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="178" priority="63" stopIfTrue="1">
+      <formula>OR($A1598="audio", $A1598="video")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="177" priority="62" stopIfTrue="1">
+      <formula>$A1598="comments"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="176" priority="61" stopIfTrue="1">
+      <formula>OR(AND(LEFT($A1598, 14)="sensor_stream ", LEN($A1598)&gt;14, NOT(ISNUMBER(SEARCH(" ", $A1598, 15)))), AND(LEFT($A1598, 17)="sensor_statistic ", LEN($A1598)&gt;17, NOT(ISNUMBER(SEARCH(" ", $A1598, 18)))))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="175" priority="79" stopIfTrue="1">
+      <formula>$A1598="begin group"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="174" priority="60" stopIfTrue="1">
+      <formula>$A1598="enumerator"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="173" priority="77" stopIfTrue="1">
       <formula>$A1598="begin repeat"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="180" priority="76" stopIfTrue="1">
+    <cfRule type="expression" dxfId="172" priority="76" stopIfTrue="1">
       <formula>$A1598="end repeat"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="179" priority="75" stopIfTrue="1">
+    <cfRule type="expression" dxfId="171" priority="75" stopIfTrue="1">
       <formula>$A1598="text"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="178" priority="74" stopIfTrue="1">
+    <cfRule type="expression" dxfId="170" priority="74" stopIfTrue="1">
       <formula>$A1598="integer"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="177" priority="73" stopIfTrue="1">
+    <cfRule type="expression" dxfId="169" priority="73" stopIfTrue="1">
       <formula>$A1598="decimal"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="176" priority="72" stopIfTrue="1">
+    <cfRule type="expression" dxfId="168" priority="72" stopIfTrue="1">
       <formula>OR(AND(LEFT($A1598, 16)="select_multiple ", LEN($A1598)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A1598, 17)))), AND(LEFT($A1598, 11)="select_one ", LEN($A1598)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A1598, 12)))))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="175" priority="71" stopIfTrue="1">
+    <cfRule type="expression" dxfId="167" priority="71" stopIfTrue="1">
       <formula>OR($A1598="username", $A1598="phonenumber", $A1598="start", $A1598="end", $A1598="deviceid", $A1598="subscriberid", $A1598="simserial", $A1598="caseid")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="174" priority="70" stopIfTrue="1">
+    <cfRule type="expression" dxfId="166" priority="70" stopIfTrue="1">
       <formula>OR($A1598="audio audit", $A1598="text audit", $A1598="speed violations count", $A1598="speed violations list", $A1598="speed violations audit")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="173" priority="69" stopIfTrue="1">
+    <cfRule type="expression" dxfId="165" priority="69" stopIfTrue="1">
       <formula>OR($A1598="geopoint", $A1598="geoshape", $A1598="geotrace")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="172" priority="68" stopIfTrue="1">
+    <cfRule type="expression" dxfId="164" priority="68" stopIfTrue="1">
       <formula>$A1598="barcode"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="171" priority="67" stopIfTrue="1">
+    <cfRule type="expression" dxfId="163" priority="67" stopIfTrue="1">
       <formula>$A1598="note"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="170" priority="66" stopIfTrue="1">
+    <cfRule type="expression" dxfId="162" priority="66" stopIfTrue="1">
       <formula>OR($A1598="calculate", $A1598="calculate_here")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="169" priority="65" stopIfTrue="1">
-      <formula>OR($A1598="date", $A1598="datetime", $A1598="time")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="168" priority="64" stopIfTrue="1">
-      <formula>$A1598="image"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="167" priority="63" stopIfTrue="1">
-      <formula>OR($A1598="audio", $A1598="video")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="166" priority="61" stopIfTrue="1">
-      <formula>OR(AND(LEFT($A1598, 14)="sensor_stream ", LEN($A1598)&gt;14, NOT(ISNUMBER(SEARCH(" ", $A1598, 15)))), AND(LEFT($A1598, 17)="sensor_statistic ", LEN($A1598)&gt;17, NOT(ISNUMBER(SEARCH(" ", $A1598, 18)))))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="165" priority="60" stopIfTrue="1">
-      <formula>$A1598="enumerator"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="164" priority="62" stopIfTrue="1">
-      <formula>$A1598="comments"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="163" priority="78" stopIfTrue="1">
-      <formula>$A1598="end group"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="162" priority="79" stopIfTrue="1">
-      <formula>$A1598="begin group"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1565">
-    <cfRule type="expression" dxfId="161" priority="297" stopIfTrue="1">
+    <cfRule type="expression" dxfId="161" priority="301" stopIfTrue="1">
+      <formula>$A1565="end group"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="160" priority="302" stopIfTrue="1">
+      <formula>$A1565="begin group"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="159" priority="303" stopIfTrue="1">
+      <formula>$A1565="image"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="158" priority="296" stopIfTrue="1">
+      <formula>$A1565="decimal"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="157" priority="288" stopIfTrue="1">
+      <formula>OR($A1565="date", $A1565="datetime")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="156" priority="289" stopIfTrue="1">
+      <formula>OR($A1565="calculate", $A1565="calculate_here")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="155" priority="290" stopIfTrue="1">
+      <formula>$A1565="note"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="154" priority="291" stopIfTrue="1">
+      <formula>$A1565="barcode"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="153" priority="292" stopIfTrue="1">
+      <formula>OR($A1565="geopoint", $A1565="geoshape", $A1565="geotrace")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="152" priority="293" stopIfTrue="1">
+      <formula>OR($A1565="audio audit", $A1565="text audit", $A1565="speed violations count", $A1565="speed violations list", $A1565="speed violations audit")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="151" priority="294" stopIfTrue="1">
+      <formula>OR($A1565="username", $A1565="phonenumber", $A1565="start", $A1565="end", $A1565="deviceid", $A1565="subscriberid", $A1565="simserial", $A1565="caseid")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="150" priority="295" stopIfTrue="1">
+      <formula>OR(AND(LEFT($A1565, 16)="select_multiple ", LEN($A1565)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A1565, 17)))), AND(LEFT($A1565, 11)="select_one ", LEN($A1565)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A1565, 12)))))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="149" priority="297" stopIfTrue="1">
       <formula>$A1565="integer"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="160" priority="298" stopIfTrue="1">
+    <cfRule type="expression" dxfId="148" priority="298" stopIfTrue="1">
       <formula>$A1565="text"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="159" priority="299" stopIfTrue="1">
+    <cfRule type="expression" dxfId="147" priority="299" stopIfTrue="1">
       <formula>$A1565="end repeat"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="158" priority="300" stopIfTrue="1">
+    <cfRule type="expression" dxfId="146" priority="300" stopIfTrue="1">
       <formula>$A1565="begin repeat"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="157" priority="301" stopIfTrue="1">
-      <formula>$A1565="end group"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="156" priority="302" stopIfTrue="1">
-      <formula>$A1565="begin group"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="155" priority="303" stopIfTrue="1">
-      <formula>$A1565="image"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="154" priority="293" stopIfTrue="1">
-      <formula>OR($A1565="audio audit", $A1565="text audit", $A1565="speed violations count", $A1565="speed violations list", $A1565="speed violations audit")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="153" priority="294" stopIfTrue="1">
-      <formula>OR($A1565="username", $A1565="phonenumber", $A1565="start", $A1565="end", $A1565="deviceid", $A1565="subscriberid", $A1565="simserial", $A1565="caseid")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="152" priority="292" stopIfTrue="1">
-      <formula>OR($A1565="geopoint", $A1565="geoshape", $A1565="geotrace")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="151" priority="291" stopIfTrue="1">
-      <formula>$A1565="barcode"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="150" priority="290" stopIfTrue="1">
-      <formula>$A1565="note"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="149" priority="289" stopIfTrue="1">
-      <formula>OR($A1565="calculate", $A1565="calculate_here")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="148" priority="288" stopIfTrue="1">
-      <formula>OR($A1565="date", $A1565="datetime")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="147" priority="295" stopIfTrue="1">
-      <formula>OR(AND(LEFT($A1565, 16)="select_multiple ", LEN($A1565)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A1565, 17)))), AND(LEFT($A1565, 11)="select_one ", LEN($A1565)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A1565, 12)))))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="146" priority="296" stopIfTrue="1">
-      <formula>$A1565="decimal"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1598">
-    <cfRule type="expression" dxfId="145" priority="165" stopIfTrue="1">
+    <cfRule type="expression" dxfId="145" priority="126" stopIfTrue="1">
+      <formula>OR($A1598="geopoint", $A1598="geoshape", $A1598="geotrace")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="144" priority="122" stopIfTrue="1">
+      <formula>$A1598="text"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="143" priority="128" stopIfTrue="1">
+      <formula>$A1598="begin group"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="142" priority="129" stopIfTrue="1">
+      <formula>$A1598="decimal"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="141" priority="130" stopIfTrue="1">
+      <formula>$A1598="integer"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="140" priority="165" stopIfTrue="1">
       <formula>$A1598="end group"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="144" priority="164" stopIfTrue="1">
-      <formula>$A1598="begin repeat"</formula>
+    <cfRule type="expression" dxfId="139" priority="123" stopIfTrue="1">
+      <formula>OR($A1598="audio", $A1598="video")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="143" priority="163" stopIfTrue="1">
+    <cfRule type="expression" dxfId="138" priority="166" stopIfTrue="1">
+      <formula>$A1598="begin group"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="137" priority="124" stopIfTrue="1">
+      <formula>$A1598="note"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="136" priority="125" stopIfTrue="1">
+      <formula>$A1598="barcode"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="135" priority="150" stopIfTrue="1">
+      <formula>OR($A1598="audio", $A1598="video")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="134" priority="151" stopIfTrue="1">
+      <formula>$A1598="image"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="133" priority="152" stopIfTrue="1">
+      <formula>OR($A1598="date", $A1598="datetime")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="132" priority="153" stopIfTrue="1">
+      <formula>OR($A1598="calculate", $A1598="calculate_here")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="131" priority="154" stopIfTrue="1">
+      <formula>$A1598="note"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="130" priority="155" stopIfTrue="1">
+      <formula>$A1598="barcode"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="129" priority="156" stopIfTrue="1">
+      <formula>OR($A1598="geopoint", $A1598="geoshape", $A1598="geotrace")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="128" priority="157" stopIfTrue="1">
+      <formula>OR($A1598="audio audit", $A1598="text audit", $A1598="speed violations count", $A1598="speed violations list", $A1598="speed violations audit")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="127" priority="158" stopIfTrue="1">
+      <formula>OR($A1598="username", $A1598="phonenumber", $A1598="start", $A1598="end", $A1598="deviceid", $A1598="subscriberid", $A1598="simserial", $A1598="caseid")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="126" priority="159" stopIfTrue="1">
+      <formula>OR(AND(LEFT($A1598, 16)="select_multiple ", LEN($A1598)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A1598, 17)))), AND(LEFT($A1598, 11)="select_one ", LEN($A1598)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A1598, 12)))))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="125" priority="160" stopIfTrue="1">
+      <formula>$A1598="decimal"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="124" priority="161" stopIfTrue="1">
+      <formula>$A1598="integer"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="123" priority="162" stopIfTrue="1">
+      <formula>$A1598="text"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="122" priority="163" stopIfTrue="1">
       <formula>$A1598="end repeat"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="142" priority="123" stopIfTrue="1">
-      <formula>OR($A1598="audio", $A1598="video")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="141" priority="124" stopIfTrue="1">
-      <formula>$A1598="note"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="140" priority="125" stopIfTrue="1">
-      <formula>$A1598="barcode"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="139" priority="126" stopIfTrue="1">
-      <formula>OR($A1598="geopoint", $A1598="geoshape", $A1598="geotrace")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="138" priority="162" stopIfTrue="1">
-      <formula>$A1598="text"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="137" priority="128" stopIfTrue="1">
-      <formula>$A1598="begin group"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="136" priority="129" stopIfTrue="1">
-      <formula>$A1598="decimal"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="135" priority="130" stopIfTrue="1">
-      <formula>$A1598="integer"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="134" priority="161" stopIfTrue="1">
-      <formula>$A1598="integer"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="133" priority="160" stopIfTrue="1">
-      <formula>$A1598="decimal"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="132" priority="156" stopIfTrue="1">
-      <formula>OR($A1598="geopoint", $A1598="geoshape", $A1598="geotrace")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="131" priority="159" stopIfTrue="1">
-      <formula>OR(AND(LEFT($A1598, 16)="select_multiple ", LEN($A1598)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A1598, 17)))), AND(LEFT($A1598, 11)="select_one ", LEN($A1598)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A1598, 12)))))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="130" priority="158" stopIfTrue="1">
-      <formula>OR($A1598="username", $A1598="phonenumber", $A1598="start", $A1598="end", $A1598="deviceid", $A1598="subscriberid", $A1598="simserial", $A1598="caseid")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="129" priority="157" stopIfTrue="1">
-      <formula>OR($A1598="audio audit", $A1598="text audit", $A1598="speed violations count", $A1598="speed violations list", $A1598="speed violations audit")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="128" priority="155" stopIfTrue="1">
-      <formula>$A1598="barcode"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="127" priority="154" stopIfTrue="1">
-      <formula>$A1598="note"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="126" priority="153" stopIfTrue="1">
-      <formula>OR($A1598="calculate", $A1598="calculate_here")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="125" priority="152" stopIfTrue="1">
-      <formula>OR($A1598="date", $A1598="datetime")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="124" priority="151" stopIfTrue="1">
-      <formula>$A1598="image"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="123" priority="150" stopIfTrue="1">
-      <formula>OR($A1598="audio", $A1598="video")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="122" priority="166" stopIfTrue="1">
-      <formula>$A1598="begin group"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="121" priority="122" stopIfTrue="1">
-      <formula>$A1598="text"</formula>
+    <cfRule type="expression" dxfId="121" priority="164" stopIfTrue="1">
+      <formula>$A1598="begin repeat"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1598:E1598 G1598">
@@ -49462,20 +49462,20 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1598:E1598 G1598:I1598 R1598:W1598">
-    <cfRule type="expression" dxfId="119" priority="181" stopIfTrue="1">
-      <formula>$A1598="text"</formula>
+    <cfRule type="expression" dxfId="119" priority="185" stopIfTrue="1">
+      <formula>$A1598="begin group"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="118" priority="182" stopIfTrue="1">
-      <formula>$A1598="end repeat"</formula>
+    <cfRule type="expression" dxfId="118" priority="184" stopIfTrue="1">
+      <formula>$A1598="end group"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="117" priority="183" stopIfTrue="1">
       <formula>$A1598="begin repeat"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="116" priority="184" stopIfTrue="1">
-      <formula>$A1598="end group"</formula>
+    <cfRule type="expression" dxfId="116" priority="182" stopIfTrue="1">
+      <formula>$A1598="end repeat"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="115" priority="185" stopIfTrue="1">
-      <formula>$A1598="begin group"</formula>
+    <cfRule type="expression" dxfId="115" priority="181" stopIfTrue="1">
+      <formula>$A1598="text"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="114" priority="180" stopIfTrue="1">
       <formula>$A1598="integer"</formula>
@@ -49488,38 +49488,38 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1598:E1598 G1598:I1598">
-    <cfRule type="expression" dxfId="111" priority="176" stopIfTrue="1">
+    <cfRule type="expression" dxfId="111" priority="172" stopIfTrue="1">
+      <formula>OR($A1598="calculate", $A1598="calculate_here")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="110" priority="173" stopIfTrue="1">
+      <formula>$A1598="note"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="109" priority="177" stopIfTrue="1">
+      <formula>OR($A1598="username", $A1598="phonenumber", $A1598="start", $A1598="end", $A1598="deviceid", $A1598="subscriberid", $A1598="simserial", $A1598="caseid")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="108" priority="176" stopIfTrue="1">
       <formula>OR($A1598="audio audit", $A1598="text audit", $A1598="speed violations count", $A1598="speed violations list", $A1598="speed violations audit")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="110" priority="175" stopIfTrue="1">
+    <cfRule type="expression" dxfId="107" priority="175" stopIfTrue="1">
       <formula>OR($A1598="geopoint", $A1598="geoshape", $A1598="geotrace")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="109" priority="174" stopIfTrue="1">
+    <cfRule type="expression" dxfId="106" priority="174" stopIfTrue="1">
       <formula>$A1598="barcode"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="108" priority="173" stopIfTrue="1">
-      <formula>$A1598="note"</formula>
+    <cfRule type="expression" dxfId="105" priority="167" stopIfTrue="1">
+      <formula>OR(AND(LEFT($A1598, 14)="sensor_stream ", LEN($A1598)&gt;14, NOT(ISNUMBER(SEARCH(" ", $A1598, 15)))), AND(LEFT($A1598, 17)="sensor_statistic ", LEN($A1598)&gt;17, NOT(ISNUMBER(SEARCH(" ", $A1598, 18)))))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="107" priority="170" stopIfTrue="1">
+    <cfRule type="expression" dxfId="104" priority="168" stopIfTrue="1">
+      <formula>$A1598="comments"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="103" priority="169" stopIfTrue="1">
+      <formula>OR($A1598="audio", $A1598="video")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="102" priority="170" stopIfTrue="1">
       <formula>$A1598="image"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="106" priority="172" stopIfTrue="1">
-      <formula>OR($A1598="calculate", $A1598="calculate_here")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="105" priority="171" stopIfTrue="1">
+    <cfRule type="expression" dxfId="101" priority="171" stopIfTrue="1">
       <formula>OR($A1598="date", $A1598="datetime")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="104" priority="167" stopIfTrue="1">
-      <formula>OR(AND(LEFT($A1598, 14)="sensor_stream ", LEN($A1598)&gt;14, NOT(ISNUMBER(SEARCH(" ", $A1598, 15)))), AND(LEFT($A1598, 17)="sensor_statistic ", LEN($A1598)&gt;17, NOT(ISNUMBER(SEARCH(" ", $A1598, 18)))))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="103" priority="168" stopIfTrue="1">
-      <formula>$A1598="comments"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="102" priority="169" stopIfTrue="1">
-      <formula>OR($A1598="audio", $A1598="video")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="101" priority="177" stopIfTrue="1">
-      <formula>OR($A1598="username", $A1598="phonenumber", $A1598="start", $A1598="end", $A1598="deviceid", $A1598="subscriberid", $A1598="simserial", $A1598="caseid")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1598:E1598">
@@ -49533,11 +49533,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E1598 G1598">
-    <cfRule type="expression" dxfId="98" priority="3" stopIfTrue="1">
+    <cfRule type="expression" dxfId="98" priority="7" stopIfTrue="1">
+      <formula>$A1598="text"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="97" priority="3" stopIfTrue="1">
       <formula>OR(AND(LEFT($A1598, 16)="select_multiple ", LEN($A1598)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A1598, 17)))), AND(LEFT($A1598, 11)="select_one ", LEN($A1598)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A1598, 12)))))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="97" priority="7" stopIfTrue="1">
-      <formula>$A1598="text"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="96" priority="2" stopIfTrue="1">
       <formula>$A1598="image"</formula>
@@ -49552,11 +49552,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1598:I1598">
-    <cfRule type="expression" dxfId="93" priority="9" stopIfTrue="1">
+    <cfRule type="expression" dxfId="93" priority="10" stopIfTrue="1">
+      <formula>$A1598="integer"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="92" priority="9" stopIfTrue="1">
       <formula>$A1598="decimal"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="92" priority="10" stopIfTrue="1">
-      <formula>$A1598="integer"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1565 P1565">
@@ -49565,17 +49565,17 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K1598:P1598">
-    <cfRule type="expression" dxfId="90" priority="42" stopIfTrue="1">
+    <cfRule type="expression" dxfId="90" priority="43" stopIfTrue="1">
+      <formula>OR($A1598="audio", $A1598="video")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="89" priority="42" stopIfTrue="1">
       <formula>$A1598="comments"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="89" priority="41" stopIfTrue="1">
+    <cfRule type="expression" dxfId="88" priority="41" stopIfTrue="1">
       <formula>OR(AND(LEFT($A1598, 14)="sensor_stream ", LEN($A1598)&gt;14, NOT(ISNUMBER(SEARCH(" ", $A1598, 15)))), AND(LEFT($A1598, 17)="sensor_statistic ", LEN($A1598)&gt;17, NOT(ISNUMBER(SEARCH(" ", $A1598, 18)))))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="88" priority="47" stopIfTrue="1">
-      <formula>$A1598="note"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="87" priority="45" stopIfTrue="1">
-      <formula>OR($A1598="date", $A1598="datetime")</formula>
+    <cfRule type="expression" dxfId="87" priority="57" stopIfTrue="1">
+      <formula>$A1598="begin repeat"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="86" priority="55" stopIfTrue="1">
       <formula>$A1598="text"</formula>
@@ -49601,26 +49601,26 @@
     <cfRule type="expression" dxfId="79" priority="48" stopIfTrue="1">
       <formula>$A1598="barcode"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="78" priority="46" stopIfTrue="1">
+    <cfRule type="expression" dxfId="78" priority="47" stopIfTrue="1">
+      <formula>$A1598="note"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="77" priority="56" stopIfTrue="1">
+      <formula>$A1598="end repeat"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="76" priority="45" stopIfTrue="1">
+      <formula>OR($A1598="date", $A1598="datetime")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="75" priority="44" stopIfTrue="1">
+      <formula>$A1598="image"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="74" priority="46" stopIfTrue="1">
       <formula>OR($A1598="calculate", $A1598="calculate_here")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="77" priority="44" stopIfTrue="1">
-      <formula>$A1598="image"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="76" priority="43" stopIfTrue="1">
-      <formula>OR($A1598="audio", $A1598="video")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="75" priority="59" stopIfTrue="1">
+    <cfRule type="expression" dxfId="73" priority="59" stopIfTrue="1">
       <formula>$A1598="begin group"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="74" priority="58" stopIfTrue="1">
+    <cfRule type="expression" dxfId="72" priority="58" stopIfTrue="1">
       <formula>$A1598="end group"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="73" priority="57" stopIfTrue="1">
-      <formula>$A1598="begin repeat"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="72" priority="56" stopIfTrue="1">
-      <formula>$A1598="end repeat"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L1597">
@@ -49632,61 +49632,61 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L1528:X1531">
-    <cfRule type="expression" dxfId="69" priority="450">
-      <formula>$A1528="end group"</formula>
+    <cfRule type="expression" dxfId="69" priority="449">
+      <formula>$A1528="integer"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="68" priority="454">
-      <formula>AND(LEFT($A1528, 10)="select_one", LEN($A1528)&gt;9)</formula>
+    <cfRule type="expression" dxfId="68" priority="448">
+      <formula>$A1528="calculate"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="67" priority="452">
-      <formula>$A1528="note"</formula>
+    <cfRule type="expression" dxfId="67" priority="447">
+      <formula>$A1528="text"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="66" priority="453">
       <formula>AND(LEFT($A1528,15)="select_multiple",LEN($A1528)&gt;14)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="65" priority="447">
-      <formula>$A1528="text"</formula>
+    <cfRule type="expression" dxfId="65" priority="450">
+      <formula>$A1528="end group"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="64" priority="448">
-      <formula>$A1528="calculate"</formula>
+    <cfRule type="expression" dxfId="64" priority="451">
+      <formula>$A1528="begin group"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="63" priority="449">
-      <formula>$A1528="integer"</formula>
+    <cfRule type="expression" dxfId="63" priority="452">
+      <formula>$A1528="note"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="62" priority="451">
-      <formula>$A1528="begin group"</formula>
+    <cfRule type="expression" dxfId="62" priority="454">
+      <formula>AND(LEFT($A1528, 10)="select_one", LEN($A1528)&gt;9)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="61" priority="446">
       <formula>$A1528="type"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L1597:X1597">
-    <cfRule type="expression" dxfId="60" priority="626">
-      <formula>AND(LEFT($A1597,15)="select_multiple",LEN($A1597)&gt;14)</formula>
+    <cfRule type="expression" dxfId="60" priority="625">
+      <formula>$A1597="note"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="59" priority="620">
-      <formula>$A1597="text"</formula>
+    <cfRule type="expression" dxfId="59" priority="624">
+      <formula>$A1597="begin group"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="58" priority="621">
-      <formula>$A1597="calculate"</formula>
+    <cfRule type="expression" dxfId="58" priority="623">
+      <formula>$A1597="end group"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="57" priority="622">
       <formula>$A1597="integer"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="56" priority="623">
-      <formula>$A1597="end group"</formula>
+    <cfRule type="expression" dxfId="56" priority="621">
+      <formula>$A1597="calculate"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="55" priority="619">
+    <cfRule type="expression" dxfId="55" priority="620">
+      <formula>$A1597="text"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="54" priority="619">
       <formula>$A1597="type"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="54" priority="624">
-      <formula>$A1597="begin group"</formula>
+    <cfRule type="expression" dxfId="53" priority="627">
+      <formula>AND(LEFT($A1597, 10)="select_one", LEN($A1597)&gt;9)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="53" priority="625">
-      <formula>$A1597="note"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="52" priority="627">
-      <formula>AND(LEFT($A1597, 10)="select_one", LEN($A1597)&gt;9)</formula>
+    <cfRule type="expression" dxfId="52" priority="626">
+      <formula>AND(LEFT($A1597,15)="select_multiple",LEN($A1597)&gt;14)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O1598">
@@ -49700,156 +49700,156 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q1565">
-    <cfRule type="expression" dxfId="49" priority="268" stopIfTrue="1">
+    <cfRule type="expression" dxfId="49" priority="273" stopIfTrue="1">
+      <formula>#REF!="barcode"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="48" priority="274" stopIfTrue="1">
+      <formula>OR(#REF!="geopoint", #REF!="geoshape", #REF!="geotrace")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="47" priority="275" stopIfTrue="1">
+      <formula>OR(#REF!="audio audit", #REF!="text audit", #REF!="speed violations count", #REF!="speed violations list", #REF!="speed violations audit")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="46" priority="276" stopIfTrue="1">
+      <formula>OR(#REF!="username", #REF!="phonenumber", #REF!="start", #REF!="end", #REF!="deviceid", #REF!="subscriberid", #REF!="simserial", #REF!="caseid")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="45" priority="277" stopIfTrue="1">
+      <formula>OR(AND(LEFT(#REF!, 16)="select_multiple ", LEN(#REF!)&gt;16, NOT(ISNUMBER(SEARCH(" ", #REF!, 17)))), AND(LEFT(#REF!, 11)="select_one ", LEN(#REF!)&gt;11, NOT(ISNUMBER(SEARCH(" ", #REF!, 12)))))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="44" priority="278" stopIfTrue="1">
+      <formula>#REF!="decimal"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="43" priority="279" stopIfTrue="1">
+      <formula>#REF!="integer"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="42" priority="281" stopIfTrue="1">
+      <formula>#REF!="end repeat"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="41" priority="282" stopIfTrue="1">
+      <formula>#REF!="begin repeat"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="40" priority="283" stopIfTrue="1">
+      <formula>#REF!="end group"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="39" priority="284" stopIfTrue="1">
+      <formula>#REF!="begin group"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="38" priority="285" stopIfTrue="1">
+      <formula>OR(AND(LEFT(#REF!, 14)="sensor_stream ", LEN(#REF!)&gt;14, NOT(ISNUMBER(SEARCH(" ", #REF!, 15)))), AND(LEFT(#REF!, 17)="sensor_statistic ", LEN(#REF!)&gt;17, NOT(ISNUMBER(SEARCH(" ", #REF!, 18)))))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="37" priority="267" stopIfTrue="1">
+      <formula>#REF!="comments"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="36" priority="280" stopIfTrue="1">
+      <formula>#REF!="text"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="35" priority="268" stopIfTrue="1">
       <formula>OR(#REF!="audio", #REF!="video")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="48" priority="279" stopIfTrue="1">
-      <formula>#REF!="integer"</formula>
+    <cfRule type="expression" dxfId="34" priority="269" stopIfTrue="1">
+      <formula>#REF!="image"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="47" priority="278" stopIfTrue="1">
-      <formula>#REF!="decimal"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="46" priority="277" stopIfTrue="1">
-      <formula>OR(AND(LEFT(#REF!, 16)="select_multiple ", LEN(#REF!)&gt;16, NOT(ISNUMBER(SEARCH(" ", #REF!, 17)))), AND(LEFT(#REF!, 11)="select_one ", LEN(#REF!)&gt;11, NOT(ISNUMBER(SEARCH(" ", #REF!, 12)))))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="45" priority="276" stopIfTrue="1">
-      <formula>OR(#REF!="username", #REF!="phonenumber", #REF!="start", #REF!="end", #REF!="deviceid", #REF!="subscriberid", #REF!="simserial", #REF!="caseid")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="44" priority="275" stopIfTrue="1">
-      <formula>OR(#REF!="audio audit", #REF!="text audit", #REF!="speed violations count", #REF!="speed violations list", #REF!="speed violations audit")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="43" priority="274" stopIfTrue="1">
-      <formula>OR(#REF!="geopoint", #REF!="geoshape", #REF!="geotrace")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="42" priority="280" stopIfTrue="1">
-      <formula>#REF!="text"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="41" priority="267" stopIfTrue="1">
-      <formula>#REF!="comments"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="40" priority="273" stopIfTrue="1">
-      <formula>#REF!="barcode"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="39" priority="271" stopIfTrue="1">
-      <formula>OR(#REF!="calculate", #REF!="calculate_here")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="38" priority="270" stopIfTrue="1">
+    <cfRule type="expression" dxfId="33" priority="270" stopIfTrue="1">
       <formula>OR(#REF!="date", #REF!="datetime")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="37" priority="269" stopIfTrue="1">
-      <formula>#REF!="image"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="36" priority="281" stopIfTrue="1">
-      <formula>#REF!="end repeat"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="35" priority="282" stopIfTrue="1">
-      <formula>#REF!="begin repeat"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="34" priority="283" stopIfTrue="1">
-      <formula>#REF!="end group"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="33" priority="284" stopIfTrue="1">
-      <formula>#REF!="begin group"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="32" priority="285" stopIfTrue="1">
-      <formula>OR(AND(LEFT(#REF!, 14)="sensor_stream ", LEN(#REF!)&gt;14, NOT(ISNUMBER(SEARCH(" ", #REF!, 15)))), AND(LEFT(#REF!, 17)="sensor_statistic ", LEN(#REF!)&gt;17, NOT(ISNUMBER(SEARCH(" ", #REF!, 18)))))</formula>
+    <cfRule type="expression" dxfId="32" priority="271" stopIfTrue="1">
+      <formula>OR(#REF!="calculate", #REF!="calculate_here")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="31" priority="272" stopIfTrue="1">
       <formula>#REF!="note"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q1598">
-    <cfRule type="expression" dxfId="30" priority="29" stopIfTrue="1">
+    <cfRule type="expression" dxfId="30" priority="40" stopIfTrue="1">
+      <formula>$A1597="begin group"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="29" priority="39" stopIfTrue="1">
+      <formula>$A1597="end group"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="28" priority="38" stopIfTrue="1">
+      <formula>$A1597="begin repeat"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="27" priority="37" stopIfTrue="1">
+      <formula>$A1597="end repeat"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="26" priority="36" stopIfTrue="1">
+      <formula>$A1597="text"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="25" priority="35" stopIfTrue="1">
+      <formula>$A1597="integer"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="24" priority="34" stopIfTrue="1">
+      <formula>$A1597="decimal"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="23" priority="33" stopIfTrue="1">
+      <formula>OR(AND(LEFT($A1597, 16)="select_multiple ", LEN($A1597)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A1597, 17)))), AND(LEFT($A1597, 11)="select_one ", LEN($A1597)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A1597, 12)))))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="22" priority="31" stopIfTrue="1">
+      <formula>OR($A1597="audio audit", $A1597="text audit", $A1597="speed violations count", $A1597="speed violations list", $A1597="speed violations audit")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="21" priority="29" stopIfTrue="1">
       <formula>$A1597="barcode"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="29" priority="30" stopIfTrue="1">
+    <cfRule type="expression" dxfId="20" priority="28" stopIfTrue="1">
+      <formula>$A1597="note"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="19" priority="27" stopIfTrue="1">
+      <formula>OR($A1597="calculate", $A1597="calculate_here")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="18" priority="30" stopIfTrue="1">
       <formula>OR($A1597="geopoint", $A1597="geoshape", $A1597="geotrace")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="28" priority="31" stopIfTrue="1">
-      <formula>OR($A1597="audio audit", $A1597="text audit", $A1597="speed violations count", $A1597="speed violations list", $A1597="speed violations audit")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="27" priority="32" stopIfTrue="1">
+    <cfRule type="expression" dxfId="17" priority="32" stopIfTrue="1">
       <formula>OR($A1597="username", $A1597="phonenumber", $A1597="start", $A1597="end", $A1597="deviceid", $A1597="subscriberid", $A1597="simserial", $A1597="caseid")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="26" priority="33" stopIfTrue="1">
-      <formula>OR(AND(LEFT($A1597, 16)="select_multiple ", LEN($A1597)&gt;16, NOT(ISNUMBER(SEARCH(" ", $A1597, 17)))), AND(LEFT($A1597, 11)="select_one ", LEN($A1597)&gt;11, NOT(ISNUMBER(SEARCH(" ", $A1597, 12)))))</formula>
+    <cfRule type="expression" dxfId="16" priority="22" stopIfTrue="1">
+      <formula>OR(AND(LEFT($A1597, 14)="sensor_stream ", LEN($A1597)&gt;14, NOT(ISNUMBER(SEARCH(" ", $A1597, 15)))), AND(LEFT($A1597, 17)="sensor_statistic ", LEN($A1597)&gt;17, NOT(ISNUMBER(SEARCH(" ", $A1597, 18)))))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="25" priority="34" stopIfTrue="1">
-      <formula>$A1597="decimal"</formula>
+    <cfRule type="expression" dxfId="15" priority="23" stopIfTrue="1">
+      <formula>$A1597="comments"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="24" priority="35" stopIfTrue="1">
-      <formula>$A1597="integer"</formula>
+    <cfRule type="expression" dxfId="14" priority="24" stopIfTrue="1">
+      <formula>OR($A1597="audio", $A1597="video")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="23" priority="36" stopIfTrue="1">
-      <formula>$A1597="text"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="22" priority="25" stopIfTrue="1">
+    <cfRule type="expression" dxfId="13" priority="25" stopIfTrue="1">
       <formula>$A1597="image"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="21" priority="39" stopIfTrue="1">
-      <formula>$A1597="end group"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="20" priority="40" stopIfTrue="1">
-      <formula>$A1597="begin group"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="19" priority="38" stopIfTrue="1">
-      <formula>$A1597="begin repeat"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="18" priority="37" stopIfTrue="1">
-      <formula>$A1597="end repeat"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="17" priority="22" stopIfTrue="1">
-      <formula>OR(AND(LEFT($A1597, 14)="sensor_stream ", LEN($A1597)&gt;14, NOT(ISNUMBER(SEARCH(" ", $A1597, 15)))), AND(LEFT($A1597, 17)="sensor_statistic ", LEN($A1597)&gt;17, NOT(ISNUMBER(SEARCH(" ", $A1597, 18)))))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="16" priority="23" stopIfTrue="1">
-      <formula>$A1597="comments"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="15" priority="24" stopIfTrue="1">
-      <formula>OR($A1597="audio", $A1597="video")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="14" priority="26" stopIfTrue="1">
+    <cfRule type="expression" dxfId="12" priority="26" stopIfTrue="1">
       <formula>OR($A1597="date", $A1597="datetime")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="13" priority="27" stopIfTrue="1">
-      <formula>OR($A1597="calculate", $A1597="calculate_here")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="12" priority="28" stopIfTrue="1">
-      <formula>$A1597="note"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R1598:W1598">
-    <cfRule type="expression" dxfId="11" priority="21" stopIfTrue="1">
-      <formula>OR($A1598="username", $A1598="phonenumber", $A1598="start", $A1598="end", $A1598="deviceid", $A1598="subscriberid", $A1598="simserial", $A1598="caseid")</formula>
+    <cfRule type="expression" dxfId="11" priority="15" stopIfTrue="1">
+      <formula>OR($A1598="date", $A1598="datetime")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="20" stopIfTrue="1">
-      <formula>OR($A1598="audio audit", $A1598="text audit", $A1598="speed violations count", $A1598="speed violations list", $A1598="speed violations audit")</formula>
+    <cfRule type="expression" dxfId="10" priority="16" stopIfTrue="1">
+      <formula>OR($A1598="calculate", $A1598="calculate_here")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="19" stopIfTrue="1">
-      <formula>OR($A1598="geopoint", $A1598="geoshape", $A1598="geotrace")</formula>
+    <cfRule type="expression" dxfId="9" priority="17" stopIfTrue="1">
+      <formula>$A1598="note"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="8" priority="18" stopIfTrue="1">
       <formula>$A1598="barcode"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="17" stopIfTrue="1">
-      <formula>$A1598="note"</formula>
+    <cfRule type="expression" dxfId="7" priority="19" stopIfTrue="1">
+      <formula>OR($A1598="geopoint", $A1598="geoshape", $A1598="geotrace")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="16" stopIfTrue="1">
-      <formula>OR($A1598="calculate", $A1598="calculate_here")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="5" priority="11" stopIfTrue="1">
+    <cfRule type="expression" dxfId="6" priority="11" stopIfTrue="1">
       <formula>OR(AND(LEFT($A1598, 14)="sensor_stream ", LEN($A1598)&gt;14, NOT(ISNUMBER(SEARCH(" ", $A1598, 15)))), AND(LEFT($A1598, 17)="sensor_statistic ", LEN($A1598)&gt;17, NOT(ISNUMBER(SEARCH(" ", $A1598, 18)))))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="12" stopIfTrue="1">
+    <cfRule type="expression" dxfId="5" priority="12" stopIfTrue="1">
       <formula>$A1598="comments"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="13" stopIfTrue="1">
+    <cfRule type="expression" dxfId="4" priority="14" stopIfTrue="1">
+      <formula>$A1598="image"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="3" priority="20" stopIfTrue="1">
+      <formula>OR($A1598="audio audit", $A1598="text audit", $A1598="speed violations count", $A1598="speed violations list", $A1598="speed violations audit")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="21" stopIfTrue="1">
+      <formula>OR($A1598="username", $A1598="phonenumber", $A1598="start", $A1598="end", $A1598="deviceid", $A1598="subscriberid", $A1598="simserial", $A1598="caseid")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="13" stopIfTrue="1">
       <formula>OR($A1598="audio", $A1598="video")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="2" priority="15" stopIfTrue="1">
-      <formula>OR($A1598="date", $A1598="datetime")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="1" priority="14" stopIfTrue="1">
-      <formula>$A1598="image"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -49858,6 +49858,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -67415,7 +67416,7 @@
       </c>
       <c r="C2" t="str">
         <f ca="1">TEXT(YEAR(NOW())-2000, "00") &amp; TEXT(MONTH(NOW()), "00") &amp; TEXT(DAY(NOW()), "00") &amp; TEXT(HOUR(NOW()), "00") &amp; TEXT(MINUTE(NOW()), "00")</f>
-        <v>2608021940</v>
+        <v>2608040700</v>
       </c>
       <c r="F2" s="11" t="s">
         <v>125</v>

</xml_diff>